<commit_message>
Narrative automatically activates or deactivates based on the presence or absence of the key; the  flag is not needed at all.
</commit_message>
<xml_diff>
--- a/reports/firm_A_report.xlsx
+++ b/reports/firm_A_report.xlsx
@@ -745,7 +745,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>(AssetClass:Structured Credit)&lt;-[:BELONGS_TO]-(Position:SC-01) | (AssetClass:High Yield Bonds)&lt;-[:BELONGS_TO]-(Position:HY-01) | (AssetClass:High Yield Bonds)&lt;-[:BELONGS_TO]-(Position:HY-02)-[:CONTRIBUTES_TO]-&gt;(Aggregate:non_ig) | sample_fund_guidelines.pdf p2 [p2_7f6467ea]</t>
+          <t>(Position:SC-01)-&gt;(AssetClass:Structured Credit) | (Position:HY-01)-&gt;(AssetClass:High Yield Bonds) | (Position:HY-02)-&gt;(AssetClass:High Yield Bonds)-[:CONTRIBUTES_TO]-&gt;(Aggregate:non_ig) | sample_fund_guidelines.pdf p2 [p2_7f6467ea]</t>
         </is>
       </c>
     </row>
@@ -819,7 +819,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>(Position:COR-03)-[:ISSUED_BY]-&gt;(Issuer:Redhill Power Pte Ltd)&lt;-[:GOVERNS]-(RiskMetric:gre_concentration) | sample_fund_guidelines.pdf p2 [p2_7f6467ea]</t>
+          <t>(Position:COR-03)-[:ISSUED_BY]-&gt;(Issuer:Redhill Power Pte Ltd) | sample_fund_guidelines.pdf p2 [p2_7f6467ea]</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>(AssetClass:Cash &amp; Cash Equivalents) | (AssetClass:MAS Bills) | (AssetClass:Singapore Government Securities) | (AssetClass:Singapore Government Securities)-[:CONTRIBUTES_TO]-&gt;(Aggregate:liquidity) | sample_fund_guidelines.pdf p2 [p2_7f6467ea]</t>
+          <t>(AssetClass:MAS Bills) | (AssetClass:Singapore Government Securities) | (AssetClass:Singapore Government Securities) | (AssetClass:Cash &amp; Cash Equivalents)-[:CONTRIBUTES_TO]-&gt;(Aggregate:liquidity) | sample_fund_guidelines.pdf p2 [p2_7f6467ea]</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>(Position:*)-[:BELONGS_TO]-&gt;(AssetClass:*) | weighted_avg(modified_duration)-&gt;(RiskMetric:modified_duration) | sample_fund_guidelines.pdf p2 [p2_7f6467ea]</t>
+          <t>(Position:*)-weighted_avg(modified_duration)-&gt;(RiskMetric:modified_duration) | sample_fund_guidelines.pdf p2 [p2_7f6467ea]</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>(Position:*) -&gt; sum(MV * duration / 10000) -&gt; (RiskMetric:dv01) | sample_fund_guidelines.pdf p2 [p2_7f6467ea]</t>
+          <t>(Position:*)-&gt;sum(MV*duration/10000)-&gt;(RiskMetric:dv01) | sample_fund_guidelines.pdf p2 [p2_7f6467ea]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
switch between list LLM model for narrative
</commit_message>
<xml_diff>
--- a/reports/firm_A_report.xlsx
+++ b/reports/firm_A_report.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Narrative" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +50,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -745,7 +750,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>(Position:SC-01)-&gt;(AssetClass:Structured Credit) | (Position:HY-01)-&gt;(AssetClass:High Yield Bonds) | (Position:HY-02)-&gt;(AssetClass:High Yield Bonds)-[:CONTRIBUTES_TO]-&gt;(Aggregate:non_ig) | sample_fund_guidelines.pdf p2 [p2_7f6467ea]</t>
+          <t>(Position:HY-01)-&gt;(AssetClass:High Yield Bonds) | (Position:HY-02)-&gt;(AssetClass:High Yield Bonds) | (Position:SC-01)-&gt;(AssetClass:Structured Credit)-[:CONTRIBUTES_TO]-&gt;(Aggregate:non_ig) | sample_fund_guidelines.pdf p2 [p2_7f6467ea]</t>
         </is>
       </c>
     </row>
@@ -856,7 +861,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>(AssetClass:MAS Bills) | (AssetClass:Singapore Government Securities) | (AssetClass:Singapore Government Securities) | (AssetClass:Cash &amp; Cash Equivalents)-[:CONTRIBUTES_TO]-&gt;(Aggregate:liquidity) | sample_fund_guidelines.pdf p2 [p2_7f6467ea]</t>
+          <t>(AssetClass:Singapore Government Securities) | (AssetClass:Singapore Government Securities) | (AssetClass:Cash &amp; Cash Equivalents) | (AssetClass:MAS Bills)-[:CONTRIBUTES_TO]-&gt;(Aggregate:liquidity) | sample_fund_guidelines.pdf p2 [p2_7f6467ea]</t>
         </is>
       </c>
     </row>
@@ -931,6 +936,37 @@
       <c r="G14" t="inlineStr">
         <is>
           <t>(Position:*)-&gt;sum(MV*duration/10000)-&gt;(RiskMetric:dv01) | sample_fund_guidelines.pdf p2 [p2_7f6467ea]</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="120" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Compliance Commentary — firm_A (LLM-generated, Gemini)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>The Meridian Fixed Income Fund remains largely compliant with regulatory requirements, maintaining a portfolio modified duration of 3.88 yrs and a portfolio dv01 of SGD 38,790 / bp. However, the fund is currently in breach of the minimum liquidity mandate, with Cash &amp; Cash Equivalents recorded at 4.0% against the required 5.0% minimum. Furthermore, the exposure to the largest_single_corporate_issuer has reached the maximum threshold of 8.0%. All other asset allocations, including the 35.0% allocation_Singapore Government Securities and 33.0% allocation_Investment Grade Corporate Bonds, remain within their respective prescribed limits.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
avoid out of memory
</commit_message>
<xml_diff>
--- a/reports/firm_A_report.xlsx
+++ b/reports/firm_A_report.xlsx
@@ -750,7 +750,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>(Position:HY-01)-&gt;(AssetClass:High Yield Bonds) | (Position:HY-02)-&gt;(AssetClass:High Yield Bonds) | (Position:SC-01)-&gt;(AssetClass:Structured Credit)-[:CONTRIBUTES_TO]-&gt;(Aggregate:non_ig) | sample_fund_guidelines.pdf p2 [p2_7f6467ea]</t>
+          <t>(Position:SC-01)-&gt;(AssetClass:Structured Credit) | (Position:HY-01)-&gt;(AssetClass:High Yield Bonds) | (Position:HY-02)-&gt;(AssetClass:High Yield Bonds)-[:CONTRIBUTES_TO]-&gt;(Aggregate:non_ig) | sample_fund_guidelines.pdf p2 [p2_7f6467ea]</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>(AssetClass:Singapore Government Securities) | (AssetClass:Singapore Government Securities) | (AssetClass:Cash &amp; Cash Equivalents) | (AssetClass:MAS Bills)-[:CONTRIBUTES_TO]-&gt;(Aggregate:liquidity) | sample_fund_guidelines.pdf p2 [p2_7f6467ea]</t>
+          <t>(AssetClass:MAS Bills) | (AssetClass:Singapore Government Securities) | (AssetClass:Singapore Government Securities) | (AssetClass:Cash &amp; Cash Equivalents)-[:CONTRIBUTES_TO]-&gt;(Aggregate:liquidity) | sample_fund_guidelines.pdf p2 [p2_7f6467ea]</t>
         </is>
       </c>
     </row>
@@ -966,7 +966,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>The Meridian Fixed Income Fund remains largely compliant with regulatory requirements, maintaining a portfolio modified duration of 3.88 yrs and a portfolio dv01 of SGD 38,790 / bp. However, the fund is currently in breach of the minimum liquidity mandate, with Cash &amp; Cash Equivalents recorded at 4.0% against the required 5.0% minimum. Furthermore, the exposure to the largest_single_corporate_issuer has reached the maximum threshold of 8.0%. All other asset allocations, including the 35.0% allocation_Singapore Government Securities and 33.0% allocation_Investment Grade Corporate Bonds, remain within their respective prescribed limits.</t>
+          <t>The Meridian Fixed Income Fund remains largely compliant with its investment mandate, maintaining a portfolio modified duration of 3.88 yrs and a portfolio dv01 of SGD 38,790 / bp. However, the fund is currently in breach of its liquidity requirements, as the allocation to Cash &amp; Cash Equivalents is 4.0% against a minimum limit of 5.0%. Furthermore, the exposure to the largest_single_corporate_issuer is currently at the maximum permitted limit of 8.0%. All other asset allocations, including the 35.0% allocation to Singapore Government Securities and 33.0% to Investment Grade Corporate Bonds, remain within their respective regulatory thresholds.</t>
         </is>
       </c>
     </row>

</xml_diff>